<commit_message>
Data Cleaning 90% Completed
</commit_message>
<xml_diff>
--- a/Excel/Section_2_Excel_Wrangling_Practice_File.xlsx
+++ b/Excel/Section_2_Excel_Wrangling_Practice_File.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Data-Analyst\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D4749B-A913-4511-A26B-7313AB15CDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27861616-CCE8-4795-880E-109AECF49937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EmployeeData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="5" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$B$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Sheet1!$B$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,8 +38,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="47">
   <si>
     <t>Full Name</t>
   </si>
@@ -151,6 +175,33 @@
   </si>
   <si>
     <t>White</t>
+  </si>
+  <si>
+    <t>Date Diff</t>
+  </si>
+  <si>
+    <t>Salary Status</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Fine</t>
+  </si>
+  <si>
+    <t>Poor</t>
+  </si>
+  <si>
+    <t>Performance</t>
   </si>
 </sst>
 </file>
@@ -212,12 +263,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -233,6 +296,926 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Project Start</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="51000"/>
+                    <a:satMod val="130000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="80000">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="93000"/>
+                    <a:satMod val="130000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="94000"/>
+                    <a:satMod val="135000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="16200000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="35000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet3!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>John Doe</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>jane smith</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>ALICE JOHNSON</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>bob Brown</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Eva White</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet3!$E$2:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45444</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3C09-4064-978C-A46082DBCC14}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Project End</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent2">
+                    <a:shade val="51000"/>
+                    <a:satMod val="130000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="80000">
+                  <a:schemeClr val="accent2">
+                    <a:shade val="93000"/>
+                    <a:satMod val="130000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent2">
+                    <a:shade val="94000"/>
+                    <a:satMod val="135000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="16200000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="35000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet3!$F$2:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>45458</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45461</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45463</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45468</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45473</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-3C09-4064-978C-A46082DBCC14}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="100"/>
+        <c:overlap val="-24"/>
+        <c:axId val="83560160"/>
+        <c:axId val="2096006432"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="83560160"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx2"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2096006432"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2096006432"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx2">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx2"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="83560160"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx2">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="207">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk2">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700">
+        <a:solidFill>
+          <a:schemeClr val="lt2"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>15875</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A075AC60-5E09-E0D1-DB45-2AB7C620E7A4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -563,6 +1546,7 @@
     <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -748,6 +1732,350 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D619080A-D8AF-4C5E-8319-37F0E7B2659F}">
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>50000</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" t="str">
+        <f>IF(C2&gt;50000,"High","Low")</f>
+        <v>Low</v>
+      </c>
+      <c r="F2" t="str" cm="1">
+        <f t="array" ref="F2">_xlfn.IFS(D2=1,"Excellent",D2=2,"Good",D2=3,"Average",D2=4,"Fine",D2=5,"Poor")</f>
+        <v>Average</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3">
+        <v>60000</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E6" si="0">IF(C3&gt;50000,"High","Low")</f>
+        <v>High</v>
+      </c>
+      <c r="F3" t="str" cm="1">
+        <f t="array" ref="F3">_xlfn.IFS(D3=1,"Excellent",D3=2,"Good",D3=3,"Average",D3=4,"Fine",D3=5,"Poor")</f>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>55000</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>High</v>
+      </c>
+      <c r="F4" t="str" cm="1">
+        <f t="array" ref="F4">_xlfn.IFS(D4=1,"Excellent",D4=2,"Good",D4=3,"Average",D4=4,"Fine",D4=5,"Poor")</f>
+        <v>Good</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5">
+        <v>45000</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>Low</v>
+      </c>
+      <c r="F5" t="str" cm="1">
+        <f t="array" ref="F5">_xlfn.IFS(D5=1,"Excellent",D5=2,"Good",D5=3,"Average",D5=4,"Fine",D5=5,"Poor")</f>
+        <v>Excellent</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6">
+        <v>70000</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>High</v>
+      </c>
+      <c r="F6" t="str" cm="1">
+        <f t="array" ref="F6">_xlfn.IFS(D6=1,"Excellent",D6=2,"Good",D6=3,"Average",D6=4,"Fine",D6=5,"Poor")</f>
+        <v>Fine</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4BA040B-BD2E-447C-9B07-041A0D90E8BC}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="4"/>
+      <c r="E1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3">
+        <v>44691</v>
+      </c>
+      <c r="C2">
+        <v>50000</v>
+      </c>
+      <c r="E2" s="3">
+        <v>45444</v>
+      </c>
+      <c r="F2" s="3">
+        <v>45458</v>
+      </c>
+      <c r="G2">
+        <f>DATEDIF(E2,F2,"d")</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3">
+        <v>44941</v>
+      </c>
+      <c r="C3">
+        <v>60000</v>
+      </c>
+      <c r="E3" s="3">
+        <v>45444</v>
+      </c>
+      <c r="F3" s="3">
+        <v>45461</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G6" si="0">DATEDIF(E3,F3,"d")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3">
+        <v>44378</v>
+      </c>
+      <c r="C4">
+        <v>55000</v>
+      </c>
+      <c r="E4" s="3">
+        <v>45444</v>
+      </c>
+      <c r="F4" s="3">
+        <v>45463</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3">
+        <v>45219</v>
+      </c>
+      <c r="C5">
+        <v>45000</v>
+      </c>
+      <c r="E5" s="3">
+        <v>45444</v>
+      </c>
+      <c r="F5" s="3">
+        <v>45468</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="3">
+        <v>43895</v>
+      </c>
+      <c r="C6">
+        <v>70000</v>
+      </c>
+      <c r="E6" s="3">
+        <v>45444</v>
+      </c>
+      <c r="F6" s="3">
+        <v>45473</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7D3A57B-792C-4DB4-94A6-5BEC9AF2EE9B}">
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -918,7 +2246,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{244A6893-5014-4948-B6FC-2D5546FEC6AB}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1005,7 +2333,7 @@
       </c>
     </row>
   </sheetData>
-  <dataConsolidate leftLabels="1" topLabels="1">
+  <dataConsolidate topLabels="1">
     <dataRefs count="1">
       <dataRef ref="A1:B6" sheet="Sheet2"/>
     </dataRefs>

</xml_diff>